<commit_message>
Engine V3 + Updated Sites
</commit_message>
<xml_diff>
--- a/output/COZY.xlsx
+++ b/output/COZY.xlsx
@@ -446,16 +446,16 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Great alexander</t>
+          <t>Divine vanilla</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Imagination by LV</t>
+          <t>Vanille Planifolia by Guerlain.</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>950</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="3">
@@ -466,16 +466,16 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Symphonic</t>
+          <t>Great alexander</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Symphony by LV</t>
+          <t>Imagination by LV</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1100</v>
+        <v>950</v>
       </c>
     </row>
     <row r="4">
@@ -506,16 +506,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>فرعون</t>
+          <t>Magnetic</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Triumph of Bacchus by Argos</t>
+          <t>La Nuit de L'Homme EDT</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1100</v>
+        <v>700</v>
       </c>
     </row>
     <row r="6">
@@ -526,12 +526,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Divine vanilla</t>
+          <t>Rebel queen</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Vanille Planifolia by Guerlain.</t>
+          <t>Voulez Vous Coucher Avec Moi</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -566,16 +566,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Magnetic</t>
+          <t>Sexy angel’s on the rocks</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>La Nuit de L'Homme EDT</t>
+          <t>angel’s share on the rocks</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>700</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="9">
@@ -586,12 +586,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Sexy angel’s on the rocks</t>
+          <t>Symphonic</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>angel’s share on the rocks</t>
+          <t>Symphony by LV</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -606,12 +606,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Rebel queen</t>
+          <t>فرعون</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Voulez Vous Coucher Avec Moi</t>
+          <t>Triumph of Bacchus by Argos</t>
         </is>
       </c>
       <c r="D10" t="n">

</xml_diff>